<commit_message>
Clean up stale Import Projects template and validation
- Sponsor was a free-text column; it now works like Owner Email --
  "Sponsor Email" resolves to an existing resource and links
  sponsor_resource_id, instead of storing a plain name with no linkage.
- Priority import validation only accepted the original four values and
  rejected "Needs prioritization", even though that's been a valid
  priority elsewhere in the app for a while -- now validates against the
  shared PRIORITIES list instead of a stale hardcoded copy.
- The template's Business Unit dropdown still listed "Corporate
  Functions" and "Human Resources", both removed from Manage Values
  since the template was made -- updated to the current list, with a
  note that these are admin-configurable and can drift over time.
- Added a Sponsor column to the import preview table so a missing/
  unlinked match is visible before committing, same as Owner already
  was.
- Instructions sheet and admin-guide.md updated to match.
</commit_message>
<xml_diff>
--- a/pmo-hub-project-import-template.xlsx
+++ b/pmo-hub-project-import-template.xlsx
@@ -167,6 +167,11 @@
     <author>PMO Hub</author>
   </authors>
   <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>If this email matches an existing PMO Hub account, the project will be linked to that person for permissions. Otherwise it is shown as text only.</t>
+      </text>
+    </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
         <t>If this email matches an existing PMO Hub account, the project will be linked to that person for permissions. Otherwise it's shown as text only.</t>
@@ -512,7 +517,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   must use one of the exact options from the list — click the cell to see the dropdown.</t>
+          <t xml:space="preserve">   must use one of the exact options from the list — click the cell to see the dropdown. Business Unit and Value Area come from Manage Values and can change over time.</t>
         </is>
       </c>
     </row>
@@ -533,14 +538,14 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>5. 'Owner Email' should match a person already set up as a resource in PMO Hub, if they have one yet.</t>
+          <t>5. 'Owner Email' and 'Sponsor Email' should each match a person already set up as a resource in PMO Hub, if they have one yet.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   If left blank or no match is found, the owner's name will show as text but won't be linked to a resource.</t>
+          <t xml:space="preserve">   If left blank or no match is found, that name shows as text only — not linked to a resource, so that person won't get edit access or see the project in their My Projects/My Capacity views.</t>
         </is>
       </c>
     </row>
@@ -657,7 +662,7 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>Sponsor Email</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
@@ -749,7 +754,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Dana Wu</t>
+          <t>dana.wu@yourcompany.com</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -824,7 +829,7 @@
   </sheetData>
   <dataValidations count="7">
     <dataValidation sqref="E3:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Corporate Functions,Customer Experience,Finance,Human Resources,Legal &amp; Compliance,Marketing,Operations,Product,Sales,Supply Chain,Technology"</formula1>
+      <formula1>"Customer Experience,Finance,Legal &amp; Compliance,Marketing,Operations,Product,Sales,Supply Chain,Technology"</formula1>
     </dataValidation>
     <dataValidation sqref="F3:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Backlog,Planned,Active,Complete,Hold"</formula1>
@@ -833,7 +838,7 @@
       <formula1>"Not Started,On Track,At Risk,Planning,Blocked,Complete"</formula1>
     </dataValidation>
     <dataValidation sqref="I3:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Critical,High,Medium,Low"</formula1>
+      <formula1>"Critical,High,Medium,Low,Needs prioritization"</formula1>
     </dataValidation>
     <dataValidation sqref="J3:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Revenue Growth,Customer Experience,Operational Efficiency,Employee Experience,Compliance &amp; Risk"</formula1>

</xml_diff>

<commit_message>
Remove Target Quarter/Target Year from Import Projects
That estimate belongs to Future Planning, not initial import -- drop
the two columns, their validation, the preview column, and the
Instructions/admin-guide text. Set it afterward on the project itself
if a Backlog row needs a rough estimate.
</commit_message>
<xml_diff>
--- a/pmo-hub-project-import-template.xlsx
+++ b/pmo-hub-project-import-template.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -580,46 +580,25 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>9. 'Target Quarter' (Q1-Q4) and 'Target Year' (e.g. 2027) are optional — use these to set a rough</t>
+          <t>9. Save this file, then upload it on the 'Import Projects' page in PMO Hub.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   estimate on a Backlog project, same as the Future Planning page. Only valid when Stage is Backlog</t>
+          <t>An example row is included on the Projects tab (row 2) — delete it before importing your real data,</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   or left blank, and both must be filled in together.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>10. Save this file, then upload it on the 'Import Projects' page in PMO Hub.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>An example row is included on the Projects tab (row 2) — delete it before importing your real data,</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
           <t>or just leave it if you're not ready and want to remove it before your final import.</t>
         </is>
       </c>
     </row>
-    <row r="22"/>
+    <row r="19"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -631,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -650,8 +629,6 @@
     <col width="40" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="26" customWidth="1" min="16" max="16"/>
-    <col width="15" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -735,16 +712,6 @@
           <t>Tags</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
-        <is>
-          <t>Target Quarter</t>
-        </is>
-      </c>
-      <c r="R1" s="3" t="inlineStr">
-        <is>
-          <t>Target Year</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -827,7 +794,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="6">
     <dataValidation sqref="E3:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Customer Experience,Finance,Legal &amp; Compliance,Marketing,Operations,Product,Sales,Supply Chain,Technology"</formula1>
     </dataValidation>
@@ -846,9 +813,6 @@
     <dataValidation sqref="H3:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Discovery,Design,Build,Testing,Deployment,Monitor"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q3:Q500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Q1,Q2,Q3,Q4"</formula1>
-    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Import Projects: derive Stage from dates, only Hold/Complete overridable
Stage was a free 5-value dropdown even though the app itself only ever
sets Backlog/Planned/Active from a project's dates (computeStageFromDates)
-- Hold and Complete are the only stages that actually require an
explicit signal. The Stage column now only accepts those two as an
override; anything else (or blank) gets computed from Start Date/Target
End Date. A Complete override also forces progress to 100 and stamps
completed_at, matching what the Mark complete action does, so an
imported completed project shows up correctly on the Completed page
and Summary's recently-completed feed instead of just carrying the
stage with none of the data that goes with it.

Template's Stage dropdown, header comment, and Instructions updated to
match, along with admin-guide.md.
</commit_message>
<xml_diff>
--- a/pmo-hub-project-import-template.xlsx
+++ b/pmo-hub-project-import-template.xlsx
@@ -167,6 +167,11 @@
     <author>PMO Hub</author>
   </authors>
   <commentList>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Leave this blank in almost every case -- PMO Hub derives Backlog/Planned/Active automatically from Start Date and Target End Date. Only enter Hold or Complete here, to mark a project as already paused or finished (something dates alone can not show).</t>
+      </text>
+    </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <t>If this email matches an existing PMO Hub account, the project will be linked to that person for permissions. Otherwise it is shown as text only.</t>
@@ -470,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -510,7 +515,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>3. Columns with a dropdown arrow (Business Unit, Stage, Status, Phase, Priority, Value Area)</t>
+          <t>3. Columns with a dropdown arrow (Business Unit, Status, Phase, Priority, Value Area)</t>
         </is>
       </c>
     </row>
@@ -552,53 +557,67 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>6. Dates should be entered as YYYY-MM-DD (e.g. 2026-03-15).</t>
+          <t>6. 'Stage' should almost always be left blank — PMO Hub derives Backlog/Planned/Active automatically from Start Date and Target End Date, the same way it does everywhere else in the app.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>7. Progress % should be a plain number from 0 to 100 (no % sign).</t>
+          <t xml:space="preserve">   Only enter Hold or Complete here, to mark a project as already paused or finished (something dates alone can not show).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>8. 'Tags' is optional — separate multiple tags with commas (e.g. 'Supply Chain, CRM System').</t>
+          <t>7. Dates should be entered as YYYY-MM-DD (e.g. 2026-03-15).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>8. Progress % should be a plain number from 0 to 100 (no % sign) — ignored and set to 100 if Stage is Complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>9. 'Tags' is optional — separate multiple tags with commas (e.g. 'Supply Chain, CRM System').</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">   A tag that doesn't exist yet will be created automatically.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>9. Save this file, then upload it on the 'Import Projects' page in PMO Hub.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>An example row is included on the Projects tab (row 2) — delete it before importing your real data,</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
+          <t>10. Save this file, then upload it on the 'Import Projects' page in PMO Hub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>An example row is included on the Projects tab (row 2) — delete it before importing your real data,</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
           <t>or just leave it if you're not ready and want to remove it before your final import.</t>
         </is>
       </c>
     </row>
-    <row r="19"/>
+    <row r="21"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -739,11 +758,6 @@
           <t>Supply Chain</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
           <t>On Track</t>
@@ -799,7 +813,7 @@
       <formula1>"Customer Experience,Finance,Legal &amp; Compliance,Marketing,Operations,Product,Sales,Supply Chain,Technology"</formula1>
     </dataValidation>
     <dataValidation sqref="F3:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Backlog,Planned,Active,Complete,Hold"</formula1>
+      <formula1>"Hold,Complete"</formula1>
     </dataValidation>
     <dataValidation sqref="G3:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,On Track,At Risk,Planning,Blocked,Complete"</formula1>

</xml_diff>